<commit_message>
Configure Supabase backend settings
</commit_message>
<xml_diff>
--- a/Prompt_Report.xlsx
+++ b/Prompt_Report.xlsx
@@ -757,10 +757,26 @@
       </c>
     </row>
     <row r="14" ht="21.95" customHeight="1" s="5">
-      <c r="A14" s="3" t="n"/>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
-      <c r="D14" s="3" t="n"/>
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Configure backend for Supabase</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Added Supabase environment settings, async SQLAlchemy database session setup, safe .env.example placeholders, and async Postgres/local SQLite dependencies.</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>mohammad</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="21.95" customHeight="1" s="5">
       <c r="A15" s="2" t="n"/>

</xml_diff>

<commit_message>
Support Supabase pooler connections
</commit_message>
<xml_diff>
--- a/Prompt_Report.xlsx
+++ b/Prompt_Report.xlsx
@@ -801,10 +801,26 @@
       </c>
     </row>
     <row r="16" ht="21.95" customHeight="1" s="5">
-      <c r="A16" s="3" t="n"/>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Fix Supabase pooler database connections</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Disabled asyncpg statement caching for Postgres pooler connections in the backend and Alembic migration engine, then ran migrations on Supabase and verified the users table.</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>mohammad</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="21.95" customHeight="1" s="5">
       <c r="A17" s="2" t="n"/>

</xml_diff>

<commit_message>
Implement JWT user authentication
</commit_message>
<xml_diff>
--- a/Prompt_Report.xlsx
+++ b/Prompt_Report.xlsx
@@ -823,10 +823,26 @@
       </c>
     </row>
     <row r="17" ht="21.95" customHeight="1" s="5">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Implement JWT user authentication</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Codex</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Added backend-owned register, login, and current-user auth with bcrypt password hashing, signed JWT access tokens, SQLAlchemy user persistence, auth routes, and focused service tests.</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>mohammad</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="21.95" customHeight="1" s="5">
       <c r="A18" s="3" t="n"/>

</xml_diff>